<commit_message>
Update figures and metrics for ICLR 2027 submission, enhancing clarity and accuracy
</commit_message>
<xml_diff>
--- a/iclr2027_submission/source_results/Results_training-20260924.xlsx
+++ b/iclr2027_submission/source_results/Results_training-20260924.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rkuiper/Documents/Code/lad-generic/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9698DC75-130D-DC4E-84D3-10CDA231B1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD03AEF-8F29-8743-9356-6C7A2DD22736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3290,7 +3290,7 @@
         <v>0.4</v>
       </c>
       <c r="N8" s="9">
-        <v>0.24</v>
+        <v>0.27200000000000002</v>
       </c>
       <c r="O8" s="9">
         <v>0.34</v>
@@ -3873,7 +3873,7 @@
       </c>
       <c r="N17" s="11">
         <f t="shared" si="2"/>
-        <v>0.51777777777777789</v>
+        <v>0.52133333333333343</v>
       </c>
       <c r="O17" s="11">
         <f t="shared" si="2"/>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="T24" s="38">
         <f ca="1">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.19999999999999996</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="25" spans="1:23">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="T25" s="38">
         <f ca="1">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.19999999999999996</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="T28" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.19999999999999996</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="29" spans="1:23">
@@ -4443,7 +4443,7 @@
       </c>
       <c r="T29" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.19999999999999996</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="30" spans="1:23">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="T31" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:23">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="T32" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.4</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="33" spans="2:28">
@@ -5327,10 +5327,10 @@
         <v>0.50891858524167999</v>
       </c>
       <c r="J53" s="26">
-        <v>0.50174209022358796</v>
+        <v>0.52174209022358797</v>
       </c>
       <c r="K53" s="26">
-        <v>0.5275748647375792</v>
+        <v>0.51757486473757897</v>
       </c>
       <c r="L53" s="26">
         <v>0.5119562703885332</v>

</xml_diff>

<commit_message>
Enhance evaluation script with diffusion and autoregressive options
- Added configuration options to enable or disable diffusion and autoregressive evaluations in `evaluate_benchmarks.py`.
- Implemented checks to ensure at least one of the evaluation methods is enabled.
- Updated logic to conditionally execute diffusion and autoregressive tasks based on the new configuration options.
- Improved output messages to reflect the status of evaluations for both methods.
- Adjusted accuracy reporting to include results from both diffusion and autoregressive evaluations.

Updated figure data and references in the ICLR 2027 submission, including:
- Modified values in `figure_data.json` for accuracy metrics.
- Added new references in `iclr2027_conference.bib`.
- Updated various figures and documents to reflect the latest results and findings.
</commit_message>
<xml_diff>
--- a/iclr2027_submission/source_results/Results_training-20260924.xlsx
+++ b/iclr2027_submission/source_results/Results_training-20260924.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rkuiper/Documents/Code/lad-generic/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD03AEF-8F29-8743-9356-6C7A2DD22736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAB3B65-4CB5-0F47-BE1B-80F7C23FAF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -272,10 +272,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 87/125 correct (0.696).</t>
         </r>
@@ -1484,16 +1483,51 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Imported from run 20260918T112818.173051Z--colab-validation
-Model: llama-3.1-8b-mask-frontier-answer90-padding10-long-epoch1-lr1e-5/checkpoint-50000
-Method: diffusion
-128 generated tokens; 32 iterations
-Mean per-answer sliding model-token Distinct-2.</t>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Imported from run 20260918T112818.173051Z--colab-validation
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Model: llama-3.1-8b-mask-frontier-answer90-padding10-long-epoch1-lr1e-5/checkpoint-50000
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Method: diffusion
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">128 generated tokens; 32 iterations
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>Mean per-answer sliding model-token Distinct-2.</t>
         </r>
       </text>
     </comment>
@@ -3289,7 +3323,7 @@
       <c r="M8" s="9">
         <v>0.4</v>
       </c>
-      <c r="N8" s="9">
+      <c r="N8" s="29">
         <v>0.27200000000000002</v>
       </c>
       <c r="O8" s="9">
@@ -3421,7 +3455,7 @@
       <c r="M10" s="9">
         <v>0.78</v>
       </c>
-      <c r="N10" s="9">
+      <c r="N10" s="29">
         <v>0.76800000000000002</v>
       </c>
       <c r="O10" s="9">
@@ -3485,8 +3519,8 @@
       <c r="M11" s="9">
         <v>0.96</v>
       </c>
-      <c r="N11" s="9">
-        <v>0.5</v>
+      <c r="N11" s="29">
+        <v>0.35199999999999998</v>
       </c>
       <c r="O11" s="9">
         <v>0.94</v>
@@ -3553,7 +3587,7 @@
       <c r="M12" s="9">
         <v>0.78</v>
       </c>
-      <c r="N12" s="9">
+      <c r="N12" s="29">
         <v>0.20799999999999999</v>
       </c>
       <c r="O12" s="9">
@@ -3621,8 +3655,8 @@
       <c r="M13" s="9">
         <v>0.82</v>
       </c>
-      <c r="N13" s="9">
-        <v>0.52</v>
+      <c r="N13" s="29">
+        <v>0.46400000000000002</v>
       </c>
       <c r="O13" s="9">
         <v>0.72</v>
@@ -3873,7 +3907,7 @@
       </c>
       <c r="N17" s="11">
         <f t="shared" si="2"/>
-        <v>0.52133333333333343</v>
+        <v>0.4986666666666667</v>
       </c>
       <c r="O17" s="11">
         <f t="shared" si="2"/>
@@ -4211,7 +4245,7 @@
       </c>
       <c r="T24" s="38">
         <f ca="1">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.8</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25" spans="1:23">
@@ -4270,7 +4304,7 @@
       </c>
       <c r="T25" s="38">
         <f ca="1">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.8</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -4296,7 +4330,7 @@
       </c>
       <c r="T26" s="38">
         <f t="shared" ref="T26:T32" ca="1" si="4">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="27" spans="1:23">
@@ -4325,7 +4359,7 @@
       </c>
       <c r="T27" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="28" spans="1:23">
@@ -4443,7 +4477,7 @@
       </c>
       <c r="T29" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-1</v>
+        <v>-0.19999999999999996</v>
       </c>
     </row>
     <row r="30" spans="1:23">
@@ -4502,7 +4536,7 @@
       </c>
       <c r="T30" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.8</v>
+        <v>-0.19999999999999996</v>
       </c>
     </row>
     <row r="31" spans="1:23">
@@ -4528,7 +4562,7 @@
       </c>
       <c r="T31" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>0</v>
+        <v>-0.19999999999999996</v>
       </c>
     </row>
     <row r="32" spans="1:23">
@@ -4556,7 +4590,7 @@
       </c>
       <c r="T32" s="38">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.8</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="33" spans="2:28">

</xml_diff>

<commit_message>
Revise abstract and results notes for accuracy; update figures and data for clarity in ICLR 2027 submission
</commit_message>
<xml_diff>
--- a/iclr2027_submission/source_results/Results_training-20260924.xlsx
+++ b/iclr2027_submission/source_results/Results_training-20260924.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rkuiper/Documents/Code/lad-generic/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAB3B65-4CB5-0F47-BE1B-80F7C23FAF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{401B61C8-CFCF-2C46-B3FE-3C732C0B7017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,10 +77,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 99/125 correct (0.792).</t>
         </r>
@@ -105,10 +104,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 108/125 correct (0.864).</t>
         </r>
@@ -174,10 +172,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 39/125 correct (0.312).</t>
         </r>
@@ -285,10 +282,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 86/125 correct (0.688).</t>
         </r>
@@ -491,10 +487,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 64/125 correct (0.512).</t>
         </r>
@@ -657,10 +652,9 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t>Imported from incomplete run 20260921T170118.455805Z--colab-validation: 38/125 correct (0.304).</t>
         </r>
@@ -788,16 +782,51 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Imported from run 20260918T112818.173051Z--colab-validation
-Model: llama-3.1-8b-mask-frontier-answer90-padding10-long-epoch1-lr1e-5/checkpoint-25000
-Method: diffusion
-128 generated tokens; 32 iterations
-Token-weighted perplexity: exp(total NLL / total scored tokens).</t>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Imported from run 20260918T112818.173051Z--colab-validation
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Model: llama-3.1-8b-mask-frontier-answer90-padding10-long-epoch1-lr1e-5/checkpoint-25000
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Method: diffusion
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">128 generated tokens; 32 iterations
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>Token-weighted perplexity: exp(total NLL / total scored tokens).</t>
         </r>
       </text>
     </comment>
@@ -1090,16 +1119,51 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Imported from run 20260918T112818.173051Z--colab-validation
-Model: gemma-2-9b-mask/best
-Method: autoregressive
-128 generated tokens; AR iterations
-Mean per-answer sliding model-token Distinct-1.</t>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Imported from run 20260918T112818.173051Z--colab-validation
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Model: gemma-2-9b-mask/best
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Method: autoregressive
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">128 generated tokens; AR iterations
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>Mean per-answer sliding model-token Distinct-1.</t>
         </r>
       </text>
     </comment>
@@ -1232,16 +1296,51 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Imported from run 20260918T112818.173051Z--colab-validation
-Model: llama-3.1-8b-mask-frontier-answer90-padding10-long-epoch1-lr1e-5/checkpoint-50000
-Method: diffusion
-128 generated tokens; 32 iterations
-Mean per-answer sliding model-token Distinct-1.</t>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Imported from run 20260918T112818.173051Z--colab-validation
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Model: llama-3.1-8b-mask-frontier-answer90-padding10-long-epoch1-lr1e-5/checkpoint-50000
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Method: diffusion
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">128 generated tokens; 32 iterations
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>Mean per-answer sliding model-token Distinct-1.</t>
         </r>
       </text>
     </comment>
@@ -1536,16 +1635,51 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Imported from run 20260918T112818.173051Z--colab-validation
-Model: llama-3.1-8b-mask/best
-Method: autoregressive
-128 generated tokens; AR iterations
-Mean per-answer sliding model-token Distinct-2.</t>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Imported from run 20260918T112818.173051Z--colab-validation
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Model: llama-3.1-8b-mask/best
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Method: autoregressive
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">128 generated tokens; AR iterations
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>Mean per-answer sliding model-token Distinct-2.</t>
         </r>
       </text>
     </comment>
@@ -1930,7 +2064,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="219">
   <si>
     <t>Blue text</t>
   </si>
@@ -3238,8 +3372,8 @@
       <c r="F7" s="28">
         <v>0.84</v>
       </c>
-      <c r="G7" s="28">
-        <v>0.79200000000000004</v>
+      <c r="G7" s="29">
+        <v>0.82399999999999995</v>
       </c>
       <c r="H7" s="9">
         <v>0.74</v>
@@ -3302,7 +3436,7 @@
       <c r="F8" s="28">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="29">
         <v>0.27200000000000002</v>
       </c>
       <c r="H8" s="9">
@@ -3366,8 +3500,8 @@
       <c r="F9" s="28">
         <v>0.63200000000000001</v>
       </c>
-      <c r="G9" s="28">
-        <v>0.56000000000000005</v>
+      <c r="G9" s="29">
+        <v>0.61599999999999999</v>
       </c>
       <c r="H9" s="9">
         <v>0.7</v>
@@ -3434,8 +3568,8 @@
       <c r="F10" s="28">
         <v>0.69599999999999995</v>
       </c>
-      <c r="G10" s="28">
-        <v>0.68799999999999994</v>
+      <c r="G10" s="29">
+        <v>0.76</v>
       </c>
       <c r="H10" s="9">
         <v>0.8</v>
@@ -3486,8 +3620,8 @@
       <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="9">
-        <v>0.38</v>
+      <c r="C11" s="29">
+        <v>0.25600000000000001</v>
       </c>
       <c r="D11" s="9">
         <v>0.74</v>
@@ -3498,8 +3632,8 @@
       <c r="F11" s="28">
         <v>0.29599999999999999</v>
       </c>
-      <c r="G11" s="28">
-        <v>0.33600000000000002</v>
+      <c r="G11" s="29">
+        <v>0.28000000000000003</v>
       </c>
       <c r="H11" s="9">
         <v>0.44</v>
@@ -3566,8 +3700,8 @@
       <c r="F12" s="28">
         <v>0.248</v>
       </c>
-      <c r="G12" s="28">
-        <v>0.216</v>
+      <c r="G12" s="29">
+        <v>0.29599999999999999</v>
       </c>
       <c r="H12" s="9">
         <v>0.34</v>
@@ -3622,8 +3756,8 @@
       <c r="B13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="9">
-        <v>0.46</v>
+      <c r="C13" s="29">
+        <v>0.36799999999999999</v>
       </c>
       <c r="D13" s="9">
         <v>0.74</v>
@@ -3634,8 +3768,8 @@
       <c r="F13" s="28">
         <v>0.41599999999999998</v>
       </c>
-      <c r="G13" s="28">
-        <v>0.51200000000000001</v>
+      <c r="G13" s="29">
+        <v>0.44</v>
       </c>
       <c r="H13" s="9">
         <v>0.4</v>
@@ -3708,8 +3842,8 @@
       <c r="F14" s="28">
         <v>0.60799999999999998</v>
       </c>
-      <c r="G14" s="28">
-        <v>0.60799999999999998</v>
+      <c r="G14" s="29">
+        <v>0.61599999999999999</v>
       </c>
       <c r="H14" s="9">
         <v>0.62</v>
@@ -3779,8 +3913,8 @@
       <c r="F15" s="28">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G15" s="28">
-        <v>0.30399999999999999</v>
+      <c r="G15" s="29">
+        <v>0.32800000000000001</v>
       </c>
       <c r="H15" s="9">
         <v>0.22</v>
@@ -3863,7 +3997,7 @@
       </c>
       <c r="C17" s="11">
         <f t="shared" ref="C17:O17" si="2">AVERAGE(C7:C15)</f>
-        <v>0.52977777777777779</v>
+        <v>0.50577777777777777</v>
       </c>
       <c r="D17" s="11">
         <f t="shared" si="2"/>
@@ -3879,7 +4013,7 @@
       </c>
       <c r="G17" s="11">
         <f t="shared" si="2"/>
-        <v>0.47644444444444445</v>
+        <v>0.49244444444444446</v>
       </c>
       <c r="H17" s="11">
         <f t="shared" si="2"/>
@@ -4188,6 +4322,12 @@
         <v>0.45180688704890121</v>
       </c>
       <c r="Q23" s="1"/>
+      <c r="R23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S23" s="2">
+        <v>0.82399999999999995</v>
+      </c>
     </row>
     <row r="24" spans="1:23">
       <c r="B24" s="7" t="s">
@@ -4236,17 +4376,13 @@
         <v>0.51374621505645135</v>
       </c>
       <c r="Q24" s="2"/>
-      <c r="R24" s="9">
-        <v>0.92</v>
-      </c>
-      <c r="S24" s="11">
-        <f>R24-0.03</f>
-        <v>0.89</v>
-      </c>
-      <c r="T24" s="38">
-        <f ca="1">ROUND(RAND()/2,1)*2-1</f>
-        <v>-1</v>
-      </c>
+      <c r="R24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S24" s="2">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="T24" s="38"/>
     </row>
     <row r="25" spans="1:23">
       <c r="B25" s="7" t="s">
@@ -4295,17 +4431,13 @@
         <v>0.53396738869179805</v>
       </c>
       <c r="Q25" s="2"/>
-      <c r="R25" s="9">
-        <v>0.4</v>
-      </c>
-      <c r="S25" s="11">
-        <f t="shared" ref="S25:S32" si="3">R25-0.03</f>
-        <v>0.37</v>
-      </c>
-      <c r="T25" s="38">
-        <f ca="1">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.6</v>
-      </c>
+      <c r="R25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S25" s="2">
+        <v>0.61599999999999999</v>
+      </c>
+      <c r="T25" s="38"/>
     </row>
     <row r="26" spans="1:23">
       <c r="E26" s="2"/>
@@ -4321,17 +4453,13 @@
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
       <c r="Q26" s="2"/>
-      <c r="R26" s="9">
-        <v>0.9</v>
-      </c>
-      <c r="S26" s="11">
-        <f t="shared" si="3"/>
-        <v>0.87</v>
-      </c>
-      <c r="T26" s="38">
-        <f t="shared" ref="T26:T32" ca="1" si="4">ROUND(RAND()/2,1)*2-1</f>
-        <v>-0.4</v>
-      </c>
+      <c r="R26" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S26" s="2">
+        <v>0.76</v>
+      </c>
+      <c r="T26" s="38"/>
     </row>
     <row r="27" spans="1:23">
       <c r="B27" s="7" t="s">
@@ -4350,17 +4478,13 @@
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
-      <c r="R27" s="9">
-        <v>0.78</v>
-      </c>
-      <c r="S27" s="11">
-        <f t="shared" si="3"/>
-        <v>0.75</v>
-      </c>
-      <c r="T27" s="38">
-        <f t="shared" ca="1" si="4"/>
-        <v>-0.6</v>
-      </c>
+      <c r="R27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S27" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="T27" s="38"/>
     </row>
     <row r="28" spans="1:23">
       <c r="B28" s="7" t="s">
@@ -4409,17 +4533,13 @@
         <v>0.74583639920375933</v>
       </c>
       <c r="Q28" s="2"/>
-      <c r="R28" s="9">
-        <v>0.96</v>
-      </c>
-      <c r="S28" s="11">
-        <f t="shared" si="3"/>
-        <v>0.92999999999999994</v>
-      </c>
-      <c r="T28" s="38">
-        <f t="shared" ca="1" si="4"/>
-        <v>-0.4</v>
-      </c>
+      <c r="R28" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="S28" s="2">
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="T28" s="38"/>
     </row>
     <row r="29" spans="1:23">
       <c r="B29" s="7" t="s">
@@ -4468,17 +4588,13 @@
         <v>0.82281252773510838</v>
       </c>
       <c r="Q29" s="2"/>
-      <c r="R29" s="9">
-        <v>0.78</v>
-      </c>
-      <c r="S29" s="11">
-        <f t="shared" si="3"/>
-        <v>0.75</v>
-      </c>
-      <c r="T29" s="38">
-        <f t="shared" ca="1" si="4"/>
-        <v>-0.19999999999999996</v>
-      </c>
+      <c r="R29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S29" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="T29" s="38"/>
     </row>
     <row r="30" spans="1:23">
       <c r="B30" s="7" t="s">
@@ -4527,17 +4643,13 @@
         <v>0.84944915824915823</v>
       </c>
       <c r="Q30" s="2"/>
-      <c r="R30" s="9">
-        <v>0.82</v>
-      </c>
-      <c r="S30" s="11">
-        <f t="shared" si="3"/>
-        <v>0.78999999999999992</v>
-      </c>
-      <c r="T30" s="38">
-        <f t="shared" ca="1" si="4"/>
-        <v>-0.19999999999999996</v>
-      </c>
+      <c r="R30" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="S30" s="2">
+        <v>0.61599999999999999</v>
+      </c>
+      <c r="T30" s="38"/>
     </row>
     <row r="31" spans="1:23">
       <c r="E31" s="2"/>
@@ -4553,17 +4665,13 @@
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
       <c r="Q31" s="2"/>
-      <c r="R31" s="9">
-        <v>0.66</v>
-      </c>
-      <c r="S31" s="11">
-        <f t="shared" si="3"/>
-        <v>0.63</v>
-      </c>
-      <c r="T31" s="38">
-        <f t="shared" ca="1" si="4"/>
-        <v>-0.19999999999999996</v>
-      </c>
+      <c r="R31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S31" s="2">
+        <v>0.32800000000000001</v>
+      </c>
+      <c r="T31" s="38"/>
     </row>
     <row r="32" spans="1:23">
       <c r="B32" s="7" t="s">
@@ -4581,17 +4689,9 @@
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
       <c r="Q32" s="2"/>
-      <c r="R32" s="9">
-        <v>0.4</v>
-      </c>
-      <c r="S32" s="11">
-        <f t="shared" si="3"/>
-        <v>0.37</v>
-      </c>
-      <c r="T32" s="38">
-        <f t="shared" ca="1" si="4"/>
-        <v>-0.6</v>
-      </c>
+      <c r="R32" s="9"/>
+      <c r="S32" s="11"/>
+      <c r="T32" s="38"/>
     </row>
     <row r="33" spans="2:28">
       <c r="B33" s="7" t="s">
@@ -8340,186 +8440,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R24">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R25">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R25">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R26">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R26">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R27">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R27">
-    <cfRule type="colorScale" priority="22">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R28">
-    <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R28">
-    <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R29">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R29">
-    <cfRule type="colorScale" priority="26">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R30">
-    <cfRule type="colorScale" priority="27">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R30">
-    <cfRule type="colorScale" priority="28">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R31">
-    <cfRule type="colorScale" priority="29">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R31">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="R32">
     <cfRule type="colorScale" priority="31">
       <colorScale>
@@ -8544,31 +8464,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R24">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R24">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R24:R32">
+  <conditionalFormatting sqref="R32">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -8580,7 +8476,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R24:R32">
+  <conditionalFormatting sqref="R32">
     <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
@@ -8592,92 +8488,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R24:R32">
+  <conditionalFormatting sqref="R32">
     <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R25">
-    <cfRule type="colorScale" priority="36">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R26">
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R27">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R28">
-    <cfRule type="colorScale" priority="39">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R29">
-    <cfRule type="colorScale" priority="40">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R30">
-    <cfRule type="colorScale" priority="41">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R31">
-    <cfRule type="colorScale" priority="42">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -8690,102 +8502,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="R32">
     <cfRule type="colorScale" priority="43">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R24">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R25">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R26">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R27">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R28">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R29">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R30">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R31">
-    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>